<commit_message>
Marcar atividade 2 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -567,13 +567,17 @@
         <v>60</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-01 21:10</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">

</xml_diff>

<commit_message>
Marcar atividade 4 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -663,13 +663,17 @@
         <v>60</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-01 21:10</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -617,13 +617,17 @@
         <v>30</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-01 22:13</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">

</xml_diff>

<commit_message>
Marcar atividade 2 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -570,14 +570,10 @@
         <v>60</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-09-01 21:10</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">

</xml_diff>

<commit_message>
Marcar atividade 5 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -713,13 +713,17 @@
         <v>40</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-02 02:03</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">

</xml_diff>

<commit_message>
Marcar atividade 471 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18661,13 +18661,17 @@
         <v>40</v>
       </c>
       <c r="I396" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K396" t="inlineStr"/>
-      <c r="L396" t="inlineStr"/>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>2026-09-02 09:59</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="n">

</xml_diff>

<commit_message>
Marcar atividade 472 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18711,13 +18711,17 @@
         <v>30</v>
       </c>
       <c r="I397" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J397" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K397" t="inlineStr"/>
-      <c r="L397" t="inlineStr"/>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>2026-09-02 11:53</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="n">

</xml_diff>

<commit_message>
Marcar atividade 472 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18714,14 +18714,10 @@
         <v>30</v>
       </c>
       <c r="J397" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K397" t="inlineStr"/>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t>2026-09-02 11:53</t>
-        </is>
-      </c>
+      <c r="L397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="n">

</xml_diff>

<commit_message>
Definir PIN inicial de Darlei
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22042,7 +22042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22066,6 +22066,11 @@
           <t>MetaSemanal</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>SenhaHash</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -22085,6 +22090,11 @@
       </c>
       <c r="D2" t="n">
         <v>14</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>03ac674216f3e15c761ee1a5e255f067953623c8b388b4459e13f978d7c846f4</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marcar atividade 471 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18664,14 +18664,10 @@
         <v>40</v>
       </c>
       <c r="J396" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K396" t="inlineStr"/>
-      <c r="L396" t="inlineStr">
-        <is>
-          <t>2026-09-02 09:59</t>
-        </is>
-      </c>
+      <c r="L396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="n">

</xml_diff>

<commit_message>
Marcar atividade 545 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22069,13 +22069,17 @@
         <v>40</v>
       </c>
       <c r="I470" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K470" t="inlineStr"/>
-      <c r="L470" t="inlineStr"/>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>2026-09-02 14:24</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" t="n">

</xml_diff>

<commit_message>
Marcar atividade 546 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22119,13 +22119,17 @@
         <v>30</v>
       </c>
       <c r="I471" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J471" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K471" t="inlineStr"/>
-      <c r="L471" t="inlineStr"/>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>2026-09-02 14:24</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" t="n">

</xml_diff>

<commit_message>
Marcar atividade 547 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22169,13 +22169,17 @@
         <v>40</v>
       </c>
       <c r="I472" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J472" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K472" t="inlineStr"/>
-      <c r="L472" t="inlineStr"/>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>2026-09-02 14:25</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" t="n">

</xml_diff>

<commit_message>
Marcar atividade 545 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22072,14 +22072,10 @@
         <v>40</v>
       </c>
       <c r="J470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K470" t="inlineStr"/>
-      <c r="L470" t="inlineStr">
-        <is>
-          <t>2026-09-02 14:24</t>
-        </is>
-      </c>
+      <c r="L470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="n">

</xml_diff>

<commit_message>
Marcar atividade 546 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22118,14 +22118,10 @@
         <v>30</v>
       </c>
       <c r="J471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K471" t="inlineStr"/>
-      <c r="L471" t="inlineStr">
-        <is>
-          <t>2026-09-02 14:24</t>
-        </is>
-      </c>
+      <c r="L471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="n">

</xml_diff>

<commit_message>
Marcar atividade 547 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -22164,14 +22164,10 @@
         <v>40</v>
       </c>
       <c r="J472" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K472" t="inlineStr"/>
-      <c r="L472" t="inlineStr">
-        <is>
-          <t>2026-09-02 14:25</t>
-        </is>
-      </c>
+      <c r="L472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="n">

</xml_diff>

<commit_message>
Migrar esquema de usuários (adicionar coluna IsAdmin)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -34002,7 +34002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34031,6 +34031,11 @@
           <t>SenhaHash</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>IsAdmin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -34056,6 +34061,9 @@
           <t>03ac674216f3e15c761ee1a5e255f067953623c8b388b4459e13f978d7c846f4</t>
         </is>
       </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -34080,6 +34088,9 @@
         <is>
           <t>9af15b336e6a9619928537df30b2e6a2376569fcf9d7e773eccede65606529a0</t>
         </is>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marcar atividade 474 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18807,13 +18807,17 @@
         <v>60</v>
       </c>
       <c r="I399" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J399" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K399" t="inlineStr"/>
-      <c r="L399" t="inlineStr"/>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>2026-09-03 10:19</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">

</xml_diff>

<commit_message>
Marcar atividade 474 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -18810,14 +18810,10 @@
         <v>60</v>
       </c>
       <c r="J399" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K399" t="inlineStr"/>
-      <c r="L399" t="inlineStr">
-        <is>
-          <t>2026-09-03 10:19</t>
-        </is>
-      </c>
+      <c r="L399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Texto com audio Mairo Vergara  (Darlei)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L469"/>
+  <dimension ref="A1:L470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22034,6 +22034,52 @@
       </c>
       <c r="K469" t="inlineStr"/>
       <c r="L469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>545</v>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Darlei</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto com audio Mairo Vergara </t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Listening</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>Mairo Vergara</t>
+        </is>
+      </c>
+      <c r="H470" t="n">
+        <v>30</v>
+      </c>
+      <c r="I470" t="n">
+        <v>0</v>
+      </c>
+      <c r="J470" t="b">
+        <v>0</v>
+      </c>
+      <c r="K470" t="inlineStr"/>
+      <c r="L470" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 1093 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -29221,13 +29221,17 @@
         <v>40</v>
       </c>
       <c r="I626" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J626" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K626" t="inlineStr"/>
-      <c r="L626" t="inlineStr"/>
+      <c r="L626" t="inlineStr">
+        <is>
+          <t>2026-09-03 14:04</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" t="n">

</xml_diff>

<commit_message>
Marcar atividade 1093 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -29224,14 +29224,10 @@
         <v>40</v>
       </c>
       <c r="J626" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K626" t="inlineStr"/>
-      <c r="L626" t="inlineStr">
-        <is>
-          <t>2026-09-03 14:04</t>
-        </is>
-      </c>
+      <c r="L626" t="inlineStr"/>
     </row>
     <row r="627">
       <c r="A627" t="n">

</xml_diff>

<commit_message>
Marcar atividade 1509 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -48357,13 +48357,17 @@
         <v>15</v>
       </c>
       <c r="I1042" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1042" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1042" t="inlineStr"/>
-      <c r="L1042" t="inlineStr"/>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>2026-09-03 14:17</t>
+        </is>
+      </c>
     </row>
     <row r="1043">
       <c r="A1043" t="n">

</xml_diff>

<commit_message>
Marcar atividade 1509 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -48360,14 +48360,10 @@
         <v>15</v>
       </c>
       <c r="J1042" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K1042" t="inlineStr"/>
-      <c r="L1042" t="inlineStr">
-        <is>
-          <t>2026-09-03 14:17</t>
-        </is>
-      </c>
+      <c r="L1042" t="inlineStr"/>
     </row>
     <row r="1043">
       <c r="A1043" t="n">

</xml_diff>

<commit_message>
Marcar atividade 469 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -517,13 +517,17 @@
         <v>30</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-03 14:54</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">

</xml_diff>

<commit_message>
Marcar atividade 470 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -567,13 +567,17 @@
         <v>20</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:02</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">

</xml_diff>

<commit_message>
Marcar atividade 473 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -717,13 +717,17 @@
         <v>30</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-04 11:06</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Assistir videos em Ingles (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1612"/>
+  <dimension ref="A1:L1613"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74604,6 +74604,52 @@
       </c>
       <c r="K1612" t="inlineStr"/>
       <c r="L1612" t="inlineStr"/>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="n">
+        <v>2080</v>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="E1613" t="inlineStr">
+        <is>
+          <t>Assistir videos em Ingles</t>
+        </is>
+      </c>
+      <c r="F1613" t="inlineStr">
+        <is>
+          <t>Listening</t>
+        </is>
+      </c>
+      <c r="G1613" t="inlineStr">
+        <is>
+          <t>Personalizado</t>
+        </is>
+      </c>
+      <c r="H1613" t="n">
+        <v>10</v>
+      </c>
+      <c r="I1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1613" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1613" t="inlineStr"/>
+      <c r="L1613" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 2080 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -74643,13 +74643,17 @@
         <v>10</v>
       </c>
       <c r="I1613" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J1613" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1613" t="inlineStr"/>
-      <c r="L1613" t="inlineStr"/>
+      <c r="L1613" t="inlineStr">
+        <is>
+          <t>2026-09-04 12:46</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adicionar atividade: English Live - Aula com professor - Venesa  (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1613"/>
+  <dimension ref="A1:L1614"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74654,6 +74654,52 @@
           <t>2026-09-04 12:46</t>
         </is>
       </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="n">
+        <v>2081</v>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="E1614" t="inlineStr">
+        <is>
+          <t xml:space="preserve">English Live - Aula com professor - Venesa </t>
+        </is>
+      </c>
+      <c r="F1614" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1614" t="inlineStr">
+        <is>
+          <t>English Live</t>
+        </is>
+      </c>
+      <c r="H1614" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1614" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1614" t="inlineStr"/>
+      <c r="L1614" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 2081 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -74693,13 +74693,17 @@
         <v>40</v>
       </c>
       <c r="I1614" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J1614" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1614" t="inlineStr"/>
-      <c r="L1614" t="inlineStr"/>
+      <c r="L1614" t="inlineStr">
+        <is>
+          <t>2026-09-04 13:49</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adicionar atividade: Aula (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1614"/>
+  <dimension ref="A1:L1615"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74704,6 +74704,52 @@
           <t>2026-09-04 13:49</t>
         </is>
       </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="n">
+        <v>2082</v>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1615" t="inlineStr">
+        <is>
+          <t>Aula</t>
+        </is>
+      </c>
+      <c r="F1615" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1615" t="inlineStr">
+        <is>
+          <t>English Live</t>
+        </is>
+      </c>
+      <c r="H1615" t="n">
+        <v>30</v>
+      </c>
+      <c r="I1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1615" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1615" t="inlineStr"/>
+      <c r="L1615" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 475 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -816,10 +816,14 @@
         <v>45</v>
       </c>
       <c r="J8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-05 02:16</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">

</xml_diff>

<commit_message>
Marcar atividade 477 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -909,13 +909,17 @@
         <v>30</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-05 09:54</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">

</xml_diff>

<commit_message>
Marcar atividade 2084 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -74843,13 +74843,17 @@
         <v>40</v>
       </c>
       <c r="I1617" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J1617" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1617" t="inlineStr"/>
-      <c r="L1617" t="inlineStr"/>
+      <c r="L1617" t="inlineStr">
+        <is>
+          <t>2026-09-05 11:01</t>
+        </is>
+      </c>
     </row>
     <row r="1618">
       <c r="A1618" t="n">

</xml_diff>

<commit_message>
Marcar atividade 2084 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -74846,14 +74846,10 @@
         <v>40</v>
       </c>
       <c r="J1617" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K1617" t="inlineStr"/>
-      <c r="L1617" t="inlineStr">
-        <is>
-          <t>2026-09-05 11:01</t>
-        </is>
-      </c>
+      <c r="L1617" t="inlineStr"/>
     </row>
     <row r="1618">
       <c r="A1618" t="n">

</xml_diff>

<commit_message>
Marcar atividade 490 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1564,13 +1564,17 @@
         <v>30</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-09 10:40</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">

</xml_diff>

<commit_message>
Marcar atividade 491 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1614,13 +1614,17 @@
         <v>20</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:09</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">

</xml_diff>

<commit_message>
Marcar atividade 492 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1664,13 +1664,17 @@
         <v>30</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:09</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">

</xml_diff>

<commit_message>
Marcar atividade 490 como pendente
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1567,14 +1567,10 @@
         <v>30</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>2026-09-09 10:40</t>
-        </is>
-      </c>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Aula De Conversação (Natália)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1570"/>
+  <dimension ref="A1:L1571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72757,6 +72757,52 @@
       </c>
       <c r="K1570" t="inlineStr"/>
       <c r="L1570" t="inlineStr"/>
+    </row>
+    <row r="1571">
+      <c r="A1571" t="n">
+        <v>3493</v>
+      </c>
+      <c r="B1571" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="C1571" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D1571" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1571" t="inlineStr">
+        <is>
+          <t>Aula De Conversação</t>
+        </is>
+      </c>
+      <c r="F1571" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1571" t="inlineStr">
+        <is>
+          <t>English Live</t>
+        </is>
+      </c>
+      <c r="H1571" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1571" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1571" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1571" t="inlineStr"/>
+      <c r="L1571" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3493 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -72796,13 +72796,17 @@
         <v>40</v>
       </c>
       <c r="I1571" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J1571" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1571" t="inlineStr"/>
-      <c r="L1571" t="inlineStr"/>
+      <c r="L1571" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:16</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adicionar atividade: Duolingo (Natália)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1571"/>
+  <dimension ref="A1:L1572"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72807,6 +72807,52 @@
           <t>2026-09-09 17:16</t>
         </is>
       </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" t="n">
+        <v>3494</v>
+      </c>
+      <c r="B1572" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="C1572" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D1572" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1572" t="inlineStr">
+        <is>
+          <t>Duolingo</t>
+        </is>
+      </c>
+      <c r="F1572" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1572" t="inlineStr">
+        <is>
+          <t>Personalizado</t>
+        </is>
+      </c>
+      <c r="H1572" t="n">
+        <v>15</v>
+      </c>
+      <c r="I1572" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1572" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1572" t="inlineStr"/>
+      <c r="L1572" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3677 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -81218,13 +81218,17 @@
         <v>15</v>
       </c>
       <c r="I1754" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1754" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1754" t="inlineStr"/>
-      <c r="L1754" t="inlineStr"/>
+      <c r="L1754" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:18</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adicionar atividade: Atividade de gramática (Natália)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1754"/>
+  <dimension ref="A1:L1755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81229,6 +81229,52 @@
           <t>2026-09-09 17:18</t>
         </is>
       </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="n">
+        <v>3678</v>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D1755" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E1755" t="inlineStr">
+        <is>
+          <t>Atividade de gramática</t>
+        </is>
+      </c>
+      <c r="F1755" t="inlineStr">
+        <is>
+          <t>Speaking</t>
+        </is>
+      </c>
+      <c r="G1755" t="inlineStr">
+        <is>
+          <t>English Live</t>
+        </is>
+      </c>
+      <c r="H1755" t="n">
+        <v>60</v>
+      </c>
+      <c r="I1755" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1755" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1755" t="inlineStr"/>
+      <c r="L1755" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3678 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -81268,13 +81268,17 @@
         <v>60</v>
       </c>
       <c r="I1755" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J1755" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1755" t="inlineStr"/>
-      <c r="L1755" t="inlineStr"/>
+      <c r="L1755" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:19</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3495 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -72846,13 +72846,17 @@
         <v>15</v>
       </c>
       <c r="I1572" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1572" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1572" t="inlineStr"/>
-      <c r="L1572" t="inlineStr"/>
+      <c r="L1572" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:29</t>
+        </is>
+      </c>
     </row>
     <row r="1573">
       <c r="A1573" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Duolingo - Uma lição (Darlei Delfino)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1755"/>
+  <dimension ref="A1:L1756"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72846,17 +72846,13 @@
         <v>15</v>
       </c>
       <c r="I1572" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J1572" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K1572" t="inlineStr"/>
-      <c r="L1572" t="inlineStr">
-        <is>
-          <t>2026-09-09 17:29</t>
-        </is>
-      </c>
+      <c r="L1572" t="inlineStr"/>
     </row>
     <row r="1573">
       <c r="A1573" t="n">
@@ -81283,6 +81279,52 @@
           <t>2026-09-09 17:19</t>
         </is>
       </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="n">
+        <v>3679</v>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>Darlei Delfino</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D1756" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E1756" t="inlineStr">
+        <is>
+          <t>Duolingo - Uma lição</t>
+        </is>
+      </c>
+      <c r="F1756" t="inlineStr">
+        <is>
+          <t>Grammar</t>
+        </is>
+      </c>
+      <c r="G1756" t="inlineStr">
+        <is>
+          <t>Personalizado</t>
+        </is>
+      </c>
+      <c r="H1756" t="n">
+        <v>10</v>
+      </c>
+      <c r="I1756" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1756" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1756" t="inlineStr"/>
+      <c r="L1756" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3679 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -81318,13 +81318,17 @@
         <v>10</v>
       </c>
       <c r="I1756" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J1756" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1756" t="inlineStr"/>
-      <c r="L1756" t="inlineStr"/>
+      <c r="L1756" t="inlineStr">
+        <is>
+          <t>2026-09-09 17:32</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 496 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1848,13 +1848,17 @@
         <v>45</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-10 11:03</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">

</xml_diff>

<commit_message>
Marcar atividade 494 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1756,13 +1756,17 @@
         <v>20</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-11 01:43</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">

</xml_diff>

<commit_message>
Marcar atividade 489 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1518,13 +1518,17 @@
         <v>20</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-11 02:58</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3203 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -59472,13 +59472,17 @@
         <v>40</v>
       </c>
       <c r="I1281" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J1281" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1281" t="inlineStr"/>
-      <c r="L1281" t="inlineStr"/>
+      <c r="L1281" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:03</t>
+        </is>
+      </c>
     </row>
     <row r="1282">
       <c r="A1282" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3204 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -59522,13 +59522,17 @@
         <v>30</v>
       </c>
       <c r="I1282" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J1282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1282" t="inlineStr"/>
-      <c r="L1282" t="inlineStr"/>
+      <c r="L1282" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:03</t>
+        </is>
+      </c>
     </row>
     <row r="1283">
       <c r="A1283" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3496 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -72920,13 +72920,17 @@
         <v>15</v>
       </c>
       <c r="I1573" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1573" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1573" t="inlineStr"/>
-      <c r="L1573" t="inlineStr"/>
+      <c r="L1573" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:03</t>
+        </is>
+      </c>
     </row>
     <row r="1574">
       <c r="A1574" t="n">

</xml_diff>

<commit_message>
Marcar atividade 3497 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -72970,13 +72970,17 @@
         <v>15</v>
       </c>
       <c r="I1574" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1574" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1574" t="inlineStr"/>
-      <c r="L1574" t="inlineStr"/>
+      <c r="L1574" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:03</t>
+        </is>
+      </c>
     </row>
     <row r="1575">
       <c r="A1575" t="n">

</xml_diff>

<commit_message>
Adicionar atividade: Leitura de Livro (Natália)
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1756"/>
+  <dimension ref="A1:L1757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -81365,6 +81365,52 @@
           <t>2026-09-09 17:32</t>
         </is>
       </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="n">
+        <v>3680</v>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>Natália</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D1757" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E1757" t="inlineStr">
+        <is>
+          <t>Leitura de Livro</t>
+        </is>
+      </c>
+      <c r="F1757" t="inlineStr">
+        <is>
+          <t>Vocabulary</t>
+        </is>
+      </c>
+      <c r="G1757" t="inlineStr">
+        <is>
+          <t>Personalizado</t>
+        </is>
+      </c>
+      <c r="H1757" t="n">
+        <v>15</v>
+      </c>
+      <c r="I1757" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1757" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1757" t="inlineStr"/>
+      <c r="L1757" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Marcar atividade 3681 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -81450,13 +81450,17 @@
         <v>15</v>
       </c>
       <c r="I1758" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J1758" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K1758" t="inlineStr"/>
-      <c r="L1758" t="inlineStr"/>
+      <c r="L1758" t="inlineStr">
+        <is>
+          <t>2026-09-11 11:12</t>
+        </is>
+      </c>
     </row>
     <row r="1759">
       <c r="A1759" t="n">

</xml_diff>

<commit_message>
Marcar atividade 493 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1714,13 +1714,17 @@
         <v>20</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-11 12:12</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">

</xml_diff>

<commit_message>
Marcar atividade 495 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -1814,13 +1814,17 @@
         <v>20</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-11 13:23</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">

</xml_diff>

<commit_message>
Marcar atividade 497 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Atividades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Usuarios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Materiais" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1914,13 +1913,17 @@
         <v>30</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-11 16:14</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -89917,186 +89920,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Usuario</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Descricao</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>URL</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>NomeArquivo</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CaminhoArquivo</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>TamanhoKB</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>DataCriacao</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Darlei Delfino</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Exercícios - Present Simple and Present Continuous</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Série de exercícios para treinar</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://www.thea.study/s/1246841602/18e468b90</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-09-06 03:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Darlei Delfino</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Vocabulary - Daily Routine</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.thea.study/s/1246892220/1d070842d</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026-09-06 04:04</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Darlei Delfino</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Jogo de Gramática</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Crie seu perfil e aceite o desafio.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://englishgrammarjourney.streamlit.app/</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2026-09-07 02:12</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Marcar atividade 499 como concluída
</commit_message>
<xml_diff>
--- a/data/estudo_ingles_dados.xlsx
+++ b/data/estudo_ingles_dados.xlsx
@@ -2009,13 +2009,17 @@
         <v>45</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-11 18:44</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">

</xml_diff>